<commit_message>
Deployed 28bb756 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/artifacts/wss_test.xlsx
+++ b/artifacts/wss_test.xlsx
@@ -609,41 +609,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>entity</t>
+          <t>expression_basis</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>property</t>
+          <t>default_unit</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>expression_basis</t>
+          <t>missing_value_code</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>default_unit</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>missing_value_code</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>label</t>
         </is>

</xml_diff>